<commit_message>
add AWS closed lost reason
</commit_message>
<xml_diff>
--- a/opportunity-samples/ACE-Data-Model.xlsx
+++ b/opportunity-samples/ACE-Data-Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mqzhu/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76BA03C-60FA-114C-841F-986ADF4833AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9E0D31-DCFA-B240-865F-084158B7B2F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7840" yWindow="1240" windowWidth="30240" windowHeight="21620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9040" yWindow="2000" windowWidth="30240" windowHeight="21620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fields" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="1359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1822" uniqueCount="1360">
   <si>
     <t>Field Description</t>
   </si>
@@ -4407,6 +4407,9 @@
 Product/Technology
 Other
 Administrative</t>
+  </si>
+  <si>
+    <t>Administrative</t>
   </si>
 </sst>
 </file>
@@ -9258,6 +9261,9 @@
       <c r="T2" s="2" t="s">
         <v>705</v>
       </c>
+      <c r="U2" s="2" t="s">
+        <v>1263</v>
+      </c>
       <c r="V2" s="1" t="s">
         <v>509</v>
       </c>
@@ -9364,6 +9370,9 @@
       </c>
       <c r="T3" s="2" t="s">
         <v>706</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>710</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>524</v>
@@ -9455,6 +9464,9 @@
       <c r="T4" s="2" t="s">
         <v>707</v>
       </c>
+      <c r="U4" s="2" t="s">
+        <v>718</v>
+      </c>
       <c r="X4" s="2" t="s">
         <v>728</v>
       </c>
@@ -9518,6 +9530,9 @@
       <c r="T5" s="2" t="s">
         <v>708</v>
       </c>
+      <c r="U5" s="2" t="s">
+        <v>709</v>
+      </c>
       <c r="X5" s="2" t="s">
         <v>729</v>
       </c>
@@ -9578,6 +9593,9 @@
       <c r="T6" s="2" t="s">
         <v>709</v>
       </c>
+      <c r="U6" s="2" t="s">
+        <v>278</v>
+      </c>
       <c r="X6" s="2" t="s">
         <v>730</v>
       </c>
@@ -9631,6 +9649,9 @@
       </c>
       <c r="T7" s="2" t="s">
         <v>1263</v>
+      </c>
+      <c r="U7" s="2" t="s">
+        <v>1359</v>
       </c>
       <c r="X7" s="2" t="s">
         <v>731</v>

</xml_diff>